<commit_message>
完成两条开发者和一条测试者的user story编写(id,name,description,notes) Complete two developer user stories and one tester user story.(id,name,description,notes)
</commit_message>
<xml_diff>
--- a/management/product backlog template.xlsx
+++ b/management/product backlog template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65E3B90D-658D-1D4D-95E4-853C40A4EE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B06739F-66FC-4F7B-8ACC-517FFB405F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Story ID</t>
   </si>
@@ -60,24 +60,79 @@
   <si>
     <t>Date finished (or planned)</t>
   </si>
+  <si>
+    <t>US-D01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Data Storage</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Developer, I want to implement a File I/O handler, so that all recruitment data is saved in .txt/csv files without using a database.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Strictly follow the project's restriction that prohibits the use of the database.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Developer, I want to create a central authentication check, so that TA, MO and admin can only get access to their own functions (like only MO can delete jobs).</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>US-D02</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Role Permission Control</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Protect system security, ensure stable functions and safeguard personal privacy.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>US-T01</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Main Workflow Test</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Tester, I want to execute an end-to-end test from registration to job application, so that I can ensure the main workflow don't have any bug.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The key step in verifying the stability of the system.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -136,8 +191,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="40% - 着色 1" xfId="1" builtinId="31"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -439,21 +494,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.1328125" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1640625" style="1"/>
+    <col min="4" max="4" width="9.1328125" style="1"/>
     <col min="5" max="5" width="28.33203125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="19.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.1640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="19.796875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.1328125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="24.796875" style="1" customWidth="1"/>
     <col min="10" max="10" width="26.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="27" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -485,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="112" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="94.5" x14ac:dyDescent="0.3">
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
@@ -493,7 +548,50 @@
         <v>7</v>
       </c>
     </row>
+    <row r="3" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="81" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="67.5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
add: 5 TA stories
</commit_message>
<xml_diff>
--- a/management/product backlog template.xlsx
+++ b/management/product backlog template.xlsx
@@ -1,96 +1,54 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{65E3B90D-658D-1D4D-95E4-853C40A4EE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="22780" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <definedNames/>
+  <calcPr calcId="122211" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>Story ID</t>
-  </si>
-  <si>
-    <t>Story Name</t>
-  </si>
-  <si>
-    <t>Acceptance Criteria</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Iteration (Sprint) number</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This is an example.
-This is a new line
-1. List 1
-2. List 2
-3. List 3
-</t>
-  </si>
-  <si>
-    <t>Estimation</t>
-  </si>
-  <si>
-    <t>This is an example.
-As a &lt;&gt;
-I want &lt;&gt;
-So that &lt;&gt;</t>
-  </si>
-  <si>
-    <t>Date started (or planned)</t>
-  </si>
-  <si>
-    <t>Date finished (or planned)</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="宋体"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <sz val="9"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.5999938962981048"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -120,35 +78,94 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="40% - 着色 1" xfId="1" builtinId="31"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -438,63 +455,275 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.796875" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="36" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1640625" style="1"/>
-    <col min="5" max="5" width="28.33203125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="19.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.1640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.33203125" style="1" customWidth="1"/>
+    <col width="9.1328125" customWidth="1" style="1" min="1" max="1"/>
+    <col width="16.6640625" customWidth="1" style="1" min="2" max="2"/>
+    <col width="36" customWidth="1" style="1" min="3" max="3"/>
+    <col width="9.1328125" customWidth="1" style="1" min="4" max="4"/>
+    <col width="28.33203125" customWidth="1" style="1" min="5" max="5"/>
+    <col width="19.796875" customWidth="1" style="1" min="6" max="7"/>
+    <col width="17.1328125" customWidth="1" style="1" min="8" max="8"/>
+    <col width="24.796875" customWidth="1" style="1" min="9" max="9"/>
+    <col width="26.33203125" customWidth="1" style="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="112" x14ac:dyDescent="0.2">
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>7</v>
+    <row r="1" ht="27" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Story ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Story Name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Iteration (Sprint) number</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Estimation</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Date started (or planned)</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Date finished (or planned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="94.5" customHeight="1">
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>This is an example.
+As a &lt;&gt;
+I want &lt;&gt;
+So that &lt;&gt;</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This is an example.
+This is a new line
+1. List 1
+2. List 2
+3. List 3
+</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="81" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>US-D01</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Data Storage</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>As a Developer, I want to implement a File I/O handler, so that all recruitment data is saved in .txt/csv files without using a database.</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>Strictly follow the project's restriction that prohibits the use of the database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="81" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>US-D02</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Role Permission Control</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>As a Developer, I want to create a central authentication check, so that TA, MO and admin can only get access to their own functions (like only MO can delete jobs).</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Protect system security, ensure stable functions and safeguard personal privacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="67.5" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>US-T01</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Main Workflow Test</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>As a Tester, I want to execute an end-to-end test from registration to job application, so that I can ensure the main workflow don't have any bug.</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>The key step in verifying the stability of the system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TA-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Create profile</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The applicant can create a personal profile in the system and fill in basic information such as student ID, programme, year of study and contact details.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Basic personal information for later applications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TA-02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Upload CV</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The applicant can upload a CV to support future job applications. The file should be easy to update if needed.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>CV upload before applying.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TA-03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>View available jobs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The applicant can view current TA vacancies in the system, including key information such as module name, requirements and deadline.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Job list with basic information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TA-04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Apply for a job</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The applicant can submit an application for a TA position through the system using the information already provided in the profile and CV.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Link application with profile and CV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TA-05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Check application status</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>The applicant can check the progress of submitted applications, for example whether an application has been received, is under review, or has a final result.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Status tracking page.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="1200" verticalDpi="1200"/>
 </worksheet>
 </file>
</xml_diff>